<commit_message>
modify: human validation ias score
</commit_message>
<xml_diff>
--- a/human_validation/judge/en/judge_D001_S003_P002__qwen3-235b.xlsx
+++ b/human_validation/judge/en/judge_D001_S003_P002__qwen3-235b.xlsx
@@ -461,6 +461,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -475,7 +476,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0.2222</v>
+        <v>0.2889</v>
       </c>
     </row>
     <row r="5">
@@ -495,7 +496,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.3333</v>
+        <v>0.4444</v>
       </c>
     </row>
     <row r="7">
@@ -505,7 +506,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="8">
@@ -558,6 +559,7 @@
         <v>0.875</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>

</xml_diff>